<commit_message>
Hide gantt cell values with number format so only fill colour shows
https://claude.ai/code/session_01HFXJ4oxyzXGQ4tLC6HuKZe
</commit_message>
<xml_diff>
--- a/Contract_Tracker.xlsx
+++ b/Contract_Tracker.xlsx
@@ -17,9 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="MM/DD/YYYY"/>
+    <numFmt numFmtId="166" formatCode=";;;"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -243,10 +244,10 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>

</xml_diff>

<commit_message>
Set gantt bar fills directly in Python so colours render on open
Conditional formatting alone wasn't reliable across Excel versions.
Fills are now written statically at generation time; conditional
formatting rules still handle live updates when Contract Data is edited.

https://claude.ai/code/session_01HFXJ4oxyzXGQ4tLC6HuKZe
</commit_message>
<xml_diff>
--- a/Contract_Tracker.xlsx
+++ b/Contract_Tracker.xlsx
@@ -202,7 +202,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -244,10 +244,17 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="5" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="9" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -267,11 +274,8 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="7">
     <dxf>
-      <font>
-        <color rgb="002E75B6"/>
-      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="002E75B6"/>
@@ -279,9 +283,20 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="0070AD47"/>
-      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00DCE6F1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="0070AD47"/>
@@ -289,9 +304,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="00ED7D31"/>
-      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00ED7D31"/>
@@ -299,9 +311,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="00FFD966"/>
-      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FFD966"/>
@@ -309,9 +318,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="009DC3E6"/>
-      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="009DC3E6"/>
@@ -1448,51 +1454,51 @@
         <f>IF(AND('Contract Data'!$E3&lt;=EOMONTH(DATE(2025,12,1),0),'Contract Data'!$F3&gt;=DATE(2025,12,1)),1,"")</f>
         <v/>
       </c>
-      <c r="R4" s="15">
+      <c r="R4" s="16">
         <f>IF(AND('Contract Data'!$E3&lt;=EOMONTH(DATE(2026,1,1),0),'Contract Data'!$F3&gt;=DATE(2026,1,1)),1,"")</f>
         <v/>
       </c>
-      <c r="S4" s="15">
+      <c r="S4" s="16">
         <f>IF(AND('Contract Data'!$E3&lt;=EOMONTH(DATE(2026,2,1),0),'Contract Data'!$F3&gt;=DATE(2026,2,1)),1,"")</f>
         <v/>
       </c>
-      <c r="T4" s="15">
+      <c r="T4" s="16">
         <f>IF(AND('Contract Data'!$E3&lt;=EOMONTH(DATE(2026,3,1),0),'Contract Data'!$F3&gt;=DATE(2026,3,1)),1,"")</f>
         <v/>
       </c>
-      <c r="U4" s="15">
+      <c r="U4" s="16">
         <f>IF(AND('Contract Data'!$E3&lt;=EOMONTH(DATE(2026,4,1),0),'Contract Data'!$F3&gt;=DATE(2026,4,1)),1,"")</f>
         <v/>
       </c>
-      <c r="V4" s="15">
+      <c r="V4" s="16">
         <f>IF(AND('Contract Data'!$E3&lt;=EOMONTH(DATE(2026,5,1),0),'Contract Data'!$F3&gt;=DATE(2026,5,1)),1,"")</f>
         <v/>
       </c>
-      <c r="W4" s="16">
+      <c r="W4" s="17">
         <f>IF(AND('Contract Data'!$E3&lt;=EOMONTH(DATE(2026,6,1),0),'Contract Data'!$F3&gt;=DATE(2026,6,1)),1,"")</f>
         <v/>
       </c>
-      <c r="X4" s="15">
+      <c r="X4" s="16">
         <f>IF(AND('Contract Data'!$E3&lt;=EOMONTH(DATE(2026,7,1),0),'Contract Data'!$F3&gt;=DATE(2026,7,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Y4" s="15">
+      <c r="Y4" s="16">
         <f>IF(AND('Contract Data'!$E3&lt;=EOMONTH(DATE(2026,8,1),0),'Contract Data'!$F3&gt;=DATE(2026,8,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Z4" s="15">
+      <c r="Z4" s="16">
         <f>IF(AND('Contract Data'!$E3&lt;=EOMONTH(DATE(2026,9,1),0),'Contract Data'!$F3&gt;=DATE(2026,9,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AA4" s="15">
+      <c r="AA4" s="16">
         <f>IF(AND('Contract Data'!$E3&lt;=EOMONTH(DATE(2026,10,1),0),'Contract Data'!$F3&gt;=DATE(2026,10,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AB4" s="15">
+      <c r="AB4" s="16">
         <f>IF(AND('Contract Data'!$E3&lt;=EOMONTH(DATE(2026,11,1),0),'Contract Data'!$F3&gt;=DATE(2026,11,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AC4" s="15">
+      <c r="AC4" s="16">
         <f>IF(AND('Contract Data'!$E3&lt;=EOMONTH(DATE(2026,12,1),0),'Contract Data'!$F3&gt;=DATE(2026,12,1)),1,"")</f>
         <v/>
       </c>
@@ -1518,99 +1524,99 @@
         <f>'Contract Data'!G4</f>
         <v/>
       </c>
-      <c r="F5" s="17">
+      <c r="F5" s="18">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2025,1,1),0),'Contract Data'!$F4&gt;=DATE(2025,1,1)),1,"")</f>
         <v/>
       </c>
-      <c r="G5" s="17">
+      <c r="G5" s="18">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2025,2,1),0),'Contract Data'!$F4&gt;=DATE(2025,2,1)),1,"")</f>
         <v/>
       </c>
-      <c r="H5" s="17">
+      <c r="H5" s="15">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2025,3,1),0),'Contract Data'!$F4&gt;=DATE(2025,3,1)),1,"")</f>
         <v/>
       </c>
-      <c r="I5" s="17">
+      <c r="I5" s="15">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2025,4,1),0),'Contract Data'!$F4&gt;=DATE(2025,4,1)),1,"")</f>
         <v/>
       </c>
-      <c r="J5" s="17">
+      <c r="J5" s="15">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2025,5,1),0),'Contract Data'!$F4&gt;=DATE(2025,5,1)),1,"")</f>
         <v/>
       </c>
-      <c r="K5" s="17">
+      <c r="K5" s="15">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2025,6,1),0),'Contract Data'!$F4&gt;=DATE(2025,6,1)),1,"")</f>
         <v/>
       </c>
-      <c r="L5" s="17">
+      <c r="L5" s="15">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2025,7,1),0),'Contract Data'!$F4&gt;=DATE(2025,7,1)),1,"")</f>
         <v/>
       </c>
-      <c r="M5" s="17">
+      <c r="M5" s="15">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2025,8,1),0),'Contract Data'!$F4&gt;=DATE(2025,8,1)),1,"")</f>
         <v/>
       </c>
-      <c r="N5" s="17">
+      <c r="N5" s="15">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2025,9,1),0),'Contract Data'!$F4&gt;=DATE(2025,9,1)),1,"")</f>
         <v/>
       </c>
-      <c r="O5" s="17">
+      <c r="O5" s="15">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2025,10,1),0),'Contract Data'!$F4&gt;=DATE(2025,10,1)),1,"")</f>
         <v/>
       </c>
-      <c r="P5" s="17">
+      <c r="P5" s="15">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2025,11,1),0),'Contract Data'!$F4&gt;=DATE(2025,11,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Q5" s="17">
+      <c r="Q5" s="15">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2025,12,1),0),'Contract Data'!$F4&gt;=DATE(2025,12,1)),1,"")</f>
         <v/>
       </c>
-      <c r="R5" s="17">
+      <c r="R5" s="15">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2026,1,1),0),'Contract Data'!$F4&gt;=DATE(2026,1,1)),1,"")</f>
         <v/>
       </c>
-      <c r="S5" s="17">
+      <c r="S5" s="15">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2026,2,1),0),'Contract Data'!$F4&gt;=DATE(2026,2,1)),1,"")</f>
         <v/>
       </c>
-      <c r="T5" s="17">
+      <c r="T5" s="18">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2026,3,1),0),'Contract Data'!$F4&gt;=DATE(2026,3,1)),1,"")</f>
         <v/>
       </c>
-      <c r="U5" s="17">
+      <c r="U5" s="18">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2026,4,1),0),'Contract Data'!$F4&gt;=DATE(2026,4,1)),1,"")</f>
         <v/>
       </c>
-      <c r="V5" s="17">
+      <c r="V5" s="18">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2026,5,1),0),'Contract Data'!$F4&gt;=DATE(2026,5,1)),1,"")</f>
         <v/>
       </c>
-      <c r="W5" s="18">
+      <c r="W5" s="19">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2026,6,1),0),'Contract Data'!$F4&gt;=DATE(2026,6,1)),1,"")</f>
         <v/>
       </c>
-      <c r="X5" s="17">
+      <c r="X5" s="18">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2026,7,1),0),'Contract Data'!$F4&gt;=DATE(2026,7,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Y5" s="17">
+      <c r="Y5" s="18">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2026,8,1),0),'Contract Data'!$F4&gt;=DATE(2026,8,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Z5" s="17">
+      <c r="Z5" s="18">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2026,9,1),0),'Contract Data'!$F4&gt;=DATE(2026,9,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AA5" s="17">
+      <c r="AA5" s="18">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2026,10,1),0),'Contract Data'!$F4&gt;=DATE(2026,10,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AB5" s="17">
+      <c r="AB5" s="18">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2026,11,1),0),'Contract Data'!$F4&gt;=DATE(2026,11,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AC5" s="17">
+      <c r="AC5" s="18">
         <f>IF(AND('Contract Data'!$E4&lt;=EOMONTH(DATE(2026,12,1),0),'Contract Data'!$F4&gt;=DATE(2026,12,1)),1,"")</f>
         <v/>
       </c>
@@ -1636,99 +1642,99 @@
         <f>'Contract Data'!G5</f>
         <v/>
       </c>
-      <c r="F6" s="15">
+      <c r="F6" s="16">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2025,1,1),0),'Contract Data'!$F5&gt;=DATE(2025,1,1)),1,"")</f>
         <v/>
       </c>
-      <c r="G6" s="15">
+      <c r="G6" s="20">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2025,2,1),0),'Contract Data'!$F5&gt;=DATE(2025,2,1)),1,"")</f>
         <v/>
       </c>
-      <c r="H6" s="15">
+      <c r="H6" s="20">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2025,3,1),0),'Contract Data'!$F5&gt;=DATE(2025,3,1)),1,"")</f>
         <v/>
       </c>
-      <c r="I6" s="15">
+      <c r="I6" s="20">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2025,4,1),0),'Contract Data'!$F5&gt;=DATE(2025,4,1)),1,"")</f>
         <v/>
       </c>
-      <c r="J6" s="15">
+      <c r="J6" s="20">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2025,5,1),0),'Contract Data'!$F5&gt;=DATE(2025,5,1)),1,"")</f>
         <v/>
       </c>
-      <c r="K6" s="15">
+      <c r="K6" s="20">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2025,6,1),0),'Contract Data'!$F5&gt;=DATE(2025,6,1)),1,"")</f>
         <v/>
       </c>
-      <c r="L6" s="15">
+      <c r="L6" s="20">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2025,7,1),0),'Contract Data'!$F5&gt;=DATE(2025,7,1)),1,"")</f>
         <v/>
       </c>
-      <c r="M6" s="15">
+      <c r="M6" s="16">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2025,8,1),0),'Contract Data'!$F5&gt;=DATE(2025,8,1)),1,"")</f>
         <v/>
       </c>
-      <c r="N6" s="15">
+      <c r="N6" s="16">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2025,9,1),0),'Contract Data'!$F5&gt;=DATE(2025,9,1)),1,"")</f>
         <v/>
       </c>
-      <c r="O6" s="15">
+      <c r="O6" s="16">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2025,10,1),0),'Contract Data'!$F5&gt;=DATE(2025,10,1)),1,"")</f>
         <v/>
       </c>
-      <c r="P6" s="15">
+      <c r="P6" s="16">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2025,11,1),0),'Contract Data'!$F5&gt;=DATE(2025,11,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Q6" s="15">
+      <c r="Q6" s="16">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2025,12,1),0),'Contract Data'!$F5&gt;=DATE(2025,12,1)),1,"")</f>
         <v/>
       </c>
-      <c r="R6" s="15">
+      <c r="R6" s="16">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2026,1,1),0),'Contract Data'!$F5&gt;=DATE(2026,1,1)),1,"")</f>
         <v/>
       </c>
-      <c r="S6" s="15">
+      <c r="S6" s="16">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2026,2,1),0),'Contract Data'!$F5&gt;=DATE(2026,2,1)),1,"")</f>
         <v/>
       </c>
-      <c r="T6" s="15">
+      <c r="T6" s="16">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2026,3,1),0),'Contract Data'!$F5&gt;=DATE(2026,3,1)),1,"")</f>
         <v/>
       </c>
-      <c r="U6" s="15">
+      <c r="U6" s="16">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2026,4,1),0),'Contract Data'!$F5&gt;=DATE(2026,4,1)),1,"")</f>
         <v/>
       </c>
-      <c r="V6" s="15">
+      <c r="V6" s="16">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2026,5,1),0),'Contract Data'!$F5&gt;=DATE(2026,5,1)),1,"")</f>
         <v/>
       </c>
-      <c r="W6" s="16">
+      <c r="W6" s="17">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2026,6,1),0),'Contract Data'!$F5&gt;=DATE(2026,6,1)),1,"")</f>
         <v/>
       </c>
-      <c r="X6" s="15">
+      <c r="X6" s="16">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2026,7,1),0),'Contract Data'!$F5&gt;=DATE(2026,7,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Y6" s="15">
+      <c r="Y6" s="16">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2026,8,1),0),'Contract Data'!$F5&gt;=DATE(2026,8,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Z6" s="15">
+      <c r="Z6" s="16">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2026,9,1),0),'Contract Data'!$F5&gt;=DATE(2026,9,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AA6" s="15">
+      <c r="AA6" s="16">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2026,10,1),0),'Contract Data'!$F5&gt;=DATE(2026,10,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AB6" s="15">
+      <c r="AB6" s="16">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2026,11,1),0),'Contract Data'!$F5&gt;=DATE(2026,11,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AC6" s="15">
+      <c r="AC6" s="16">
         <f>IF(AND('Contract Data'!$E5&lt;=EOMONTH(DATE(2026,12,1),0),'Contract Data'!$F5&gt;=DATE(2026,12,1)),1,"")</f>
         <v/>
       </c>
@@ -1754,99 +1760,99 @@
         <f>'Contract Data'!G6</f>
         <v/>
       </c>
-      <c r="F7" s="17">
+      <c r="F7" s="18">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2025,1,1),0),'Contract Data'!$F6&gt;=DATE(2025,1,1)),1,"")</f>
         <v/>
       </c>
-      <c r="G7" s="17">
+      <c r="G7" s="18">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2025,2,1),0),'Contract Data'!$F6&gt;=DATE(2025,2,1)),1,"")</f>
         <v/>
       </c>
-      <c r="H7" s="17">
+      <c r="H7" s="18">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2025,3,1),0),'Contract Data'!$F6&gt;=DATE(2025,3,1)),1,"")</f>
         <v/>
       </c>
-      <c r="I7" s="17">
+      <c r="I7" s="18">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2025,4,1),0),'Contract Data'!$F6&gt;=DATE(2025,4,1)),1,"")</f>
         <v/>
       </c>
-      <c r="J7" s="17">
+      <c r="J7" s="18">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2025,5,1),0),'Contract Data'!$F6&gt;=DATE(2025,5,1)),1,"")</f>
         <v/>
       </c>
-      <c r="K7" s="17">
+      <c r="K7" s="20">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2025,6,1),0),'Contract Data'!$F6&gt;=DATE(2025,6,1)),1,"")</f>
         <v/>
       </c>
-      <c r="L7" s="17">
+      <c r="L7" s="20">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2025,7,1),0),'Contract Data'!$F6&gt;=DATE(2025,7,1)),1,"")</f>
         <v/>
       </c>
-      <c r="M7" s="17">
+      <c r="M7" s="20">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2025,8,1),0),'Contract Data'!$F6&gt;=DATE(2025,8,1)),1,"")</f>
         <v/>
       </c>
-      <c r="N7" s="17">
+      <c r="N7" s="20">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2025,9,1),0),'Contract Data'!$F6&gt;=DATE(2025,9,1)),1,"")</f>
         <v/>
       </c>
-      <c r="O7" s="17">
+      <c r="O7" s="20">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2025,10,1),0),'Contract Data'!$F6&gt;=DATE(2025,10,1)),1,"")</f>
         <v/>
       </c>
-      <c r="P7" s="17">
+      <c r="P7" s="20">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2025,11,1),0),'Contract Data'!$F6&gt;=DATE(2025,11,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Q7" s="17">
+      <c r="Q7" s="20">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2025,12,1),0),'Contract Data'!$F6&gt;=DATE(2025,12,1)),1,"")</f>
         <v/>
       </c>
-      <c r="R7" s="17">
+      <c r="R7" s="20">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2026,1,1),0),'Contract Data'!$F6&gt;=DATE(2026,1,1)),1,"")</f>
         <v/>
       </c>
-      <c r="S7" s="17">
+      <c r="S7" s="20">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2026,2,1),0),'Contract Data'!$F6&gt;=DATE(2026,2,1)),1,"")</f>
         <v/>
       </c>
-      <c r="T7" s="17">
+      <c r="T7" s="20">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2026,3,1),0),'Contract Data'!$F6&gt;=DATE(2026,3,1)),1,"")</f>
         <v/>
       </c>
-      <c r="U7" s="17">
+      <c r="U7" s="20">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2026,4,1),0),'Contract Data'!$F6&gt;=DATE(2026,4,1)),1,"")</f>
         <v/>
       </c>
-      <c r="V7" s="17">
+      <c r="V7" s="20">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2026,5,1),0),'Contract Data'!$F6&gt;=DATE(2026,5,1)),1,"")</f>
         <v/>
       </c>
-      <c r="W7" s="18">
+      <c r="W7" s="19">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2026,6,1),0),'Contract Data'!$F6&gt;=DATE(2026,6,1)),1,"")</f>
         <v/>
       </c>
-      <c r="X7" s="17">
+      <c r="X7" s="18">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2026,7,1),0),'Contract Data'!$F6&gt;=DATE(2026,7,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Y7" s="17">
+      <c r="Y7" s="18">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2026,8,1),0),'Contract Data'!$F6&gt;=DATE(2026,8,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Z7" s="17">
+      <c r="Z7" s="18">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2026,9,1),0),'Contract Data'!$F6&gt;=DATE(2026,9,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AA7" s="17">
+      <c r="AA7" s="18">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2026,10,1),0),'Contract Data'!$F6&gt;=DATE(2026,10,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AB7" s="17">
+      <c r="AB7" s="18">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2026,11,1),0),'Contract Data'!$F6&gt;=DATE(2026,11,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AC7" s="17">
+      <c r="AC7" s="18">
         <f>IF(AND('Contract Data'!$E6&lt;=EOMONTH(DATE(2026,12,1),0),'Contract Data'!$F6&gt;=DATE(2026,12,1)),1,"")</f>
         <v/>
       </c>
@@ -1872,99 +1878,99 @@
         <f>'Contract Data'!G7</f>
         <v/>
       </c>
-      <c r="F8" s="15">
+      <c r="F8" s="16">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2025,1,1),0),'Contract Data'!$F7&gt;=DATE(2025,1,1)),1,"")</f>
         <v/>
       </c>
-      <c r="G8" s="15">
+      <c r="G8" s="16">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2025,2,1),0),'Contract Data'!$F7&gt;=DATE(2025,2,1)),1,"")</f>
         <v/>
       </c>
-      <c r="H8" s="15">
+      <c r="H8" s="16">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2025,3,1),0),'Contract Data'!$F7&gt;=DATE(2025,3,1)),1,"")</f>
         <v/>
       </c>
-      <c r="I8" s="15">
+      <c r="I8" s="21">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2025,4,1),0),'Contract Data'!$F7&gt;=DATE(2025,4,1)),1,"")</f>
         <v/>
       </c>
-      <c r="J8" s="15">
+      <c r="J8" s="21">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2025,5,1),0),'Contract Data'!$F7&gt;=DATE(2025,5,1)),1,"")</f>
         <v/>
       </c>
-      <c r="K8" s="15">
+      <c r="K8" s="21">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2025,6,1),0),'Contract Data'!$F7&gt;=DATE(2025,6,1)),1,"")</f>
         <v/>
       </c>
-      <c r="L8" s="15">
+      <c r="L8" s="21">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2025,7,1),0),'Contract Data'!$F7&gt;=DATE(2025,7,1)),1,"")</f>
         <v/>
       </c>
-      <c r="M8" s="15">
+      <c r="M8" s="21">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2025,8,1),0),'Contract Data'!$F7&gt;=DATE(2025,8,1)),1,"")</f>
         <v/>
       </c>
-      <c r="N8" s="15">
+      <c r="N8" s="21">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2025,9,1),0),'Contract Data'!$F7&gt;=DATE(2025,9,1)),1,"")</f>
         <v/>
       </c>
-      <c r="O8" s="15">
+      <c r="O8" s="16">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2025,10,1),0),'Contract Data'!$F7&gt;=DATE(2025,10,1)),1,"")</f>
         <v/>
       </c>
-      <c r="P8" s="15">
+      <c r="P8" s="16">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2025,11,1),0),'Contract Data'!$F7&gt;=DATE(2025,11,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Q8" s="15">
+      <c r="Q8" s="16">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2025,12,1),0),'Contract Data'!$F7&gt;=DATE(2025,12,1)),1,"")</f>
         <v/>
       </c>
-      <c r="R8" s="15">
+      <c r="R8" s="16">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2026,1,1),0),'Contract Data'!$F7&gt;=DATE(2026,1,1)),1,"")</f>
         <v/>
       </c>
-      <c r="S8" s="15">
+      <c r="S8" s="16">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2026,2,1),0),'Contract Data'!$F7&gt;=DATE(2026,2,1)),1,"")</f>
         <v/>
       </c>
-      <c r="T8" s="15">
+      <c r="T8" s="16">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2026,3,1),0),'Contract Data'!$F7&gt;=DATE(2026,3,1)),1,"")</f>
         <v/>
       </c>
-      <c r="U8" s="15">
+      <c r="U8" s="16">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2026,4,1),0),'Contract Data'!$F7&gt;=DATE(2026,4,1)),1,"")</f>
         <v/>
       </c>
-      <c r="V8" s="15">
+      <c r="V8" s="16">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2026,5,1),0),'Contract Data'!$F7&gt;=DATE(2026,5,1)),1,"")</f>
         <v/>
       </c>
-      <c r="W8" s="16">
+      <c r="W8" s="17">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2026,6,1),0),'Contract Data'!$F7&gt;=DATE(2026,6,1)),1,"")</f>
         <v/>
       </c>
-      <c r="X8" s="15">
+      <c r="X8" s="16">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2026,7,1),0),'Contract Data'!$F7&gt;=DATE(2026,7,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Y8" s="15">
+      <c r="Y8" s="16">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2026,8,1),0),'Contract Data'!$F7&gt;=DATE(2026,8,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Z8" s="15">
+      <c r="Z8" s="16">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2026,9,1),0),'Contract Data'!$F7&gt;=DATE(2026,9,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AA8" s="15">
+      <c r="AA8" s="16">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2026,10,1),0),'Contract Data'!$F7&gt;=DATE(2026,10,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AB8" s="15">
+      <c r="AB8" s="16">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2026,11,1),0),'Contract Data'!$F7&gt;=DATE(2026,11,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AC8" s="15">
+      <c r="AC8" s="16">
         <f>IF(AND('Contract Data'!$E7&lt;=EOMONTH(DATE(2026,12,1),0),'Contract Data'!$F7&gt;=DATE(2026,12,1)),1,"")</f>
         <v/>
       </c>
@@ -1990,99 +1996,99 @@
         <f>'Contract Data'!G8</f>
         <v/>
       </c>
-      <c r="F9" s="17">
+      <c r="F9" s="18">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2025,1,1),0),'Contract Data'!$F8&gt;=DATE(2025,1,1)),1,"")</f>
         <v/>
       </c>
-      <c r="G9" s="17">
+      <c r="G9" s="18">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2025,2,1),0),'Contract Data'!$F8&gt;=DATE(2025,2,1)),1,"")</f>
         <v/>
       </c>
-      <c r="H9" s="17">
+      <c r="H9" s="18">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2025,3,1),0),'Contract Data'!$F8&gt;=DATE(2025,3,1)),1,"")</f>
         <v/>
       </c>
-      <c r="I9" s="17">
+      <c r="I9" s="18">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2025,4,1),0),'Contract Data'!$F8&gt;=DATE(2025,4,1)),1,"")</f>
         <v/>
       </c>
-      <c r="J9" s="17">
+      <c r="J9" s="18">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2025,5,1),0),'Contract Data'!$F8&gt;=DATE(2025,5,1)),1,"")</f>
         <v/>
       </c>
-      <c r="K9" s="17">
+      <c r="K9" s="18">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2025,6,1),0),'Contract Data'!$F8&gt;=DATE(2025,6,1)),1,"")</f>
         <v/>
       </c>
-      <c r="L9" s="17">
+      <c r="L9" s="18">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2025,7,1),0),'Contract Data'!$F8&gt;=DATE(2025,7,1)),1,"")</f>
         <v/>
       </c>
-      <c r="M9" s="17">
+      <c r="M9" s="18">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2025,8,1),0),'Contract Data'!$F8&gt;=DATE(2025,8,1)),1,"")</f>
         <v/>
       </c>
-      <c r="N9" s="17">
+      <c r="N9" s="21">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2025,9,1),0),'Contract Data'!$F8&gt;=DATE(2025,9,1)),1,"")</f>
         <v/>
       </c>
-      <c r="O9" s="17">
+      <c r="O9" s="21">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2025,10,1),0),'Contract Data'!$F8&gt;=DATE(2025,10,1)),1,"")</f>
         <v/>
       </c>
-      <c r="P9" s="17">
+      <c r="P9" s="21">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2025,11,1),0),'Contract Data'!$F8&gt;=DATE(2025,11,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Q9" s="17">
+      <c r="Q9" s="21">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2025,12,1),0),'Contract Data'!$F8&gt;=DATE(2025,12,1)),1,"")</f>
         <v/>
       </c>
-      <c r="R9" s="17">
+      <c r="R9" s="21">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2026,1,1),0),'Contract Data'!$F8&gt;=DATE(2026,1,1)),1,"")</f>
         <v/>
       </c>
-      <c r="S9" s="17">
+      <c r="S9" s="21">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2026,2,1),0),'Contract Data'!$F8&gt;=DATE(2026,2,1)),1,"")</f>
         <v/>
       </c>
-      <c r="T9" s="17">
+      <c r="T9" s="21">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2026,3,1),0),'Contract Data'!$F8&gt;=DATE(2026,3,1)),1,"")</f>
         <v/>
       </c>
-      <c r="U9" s="17">
+      <c r="U9" s="21">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2026,4,1),0),'Contract Data'!$F8&gt;=DATE(2026,4,1)),1,"")</f>
         <v/>
       </c>
-      <c r="V9" s="17">
+      <c r="V9" s="21">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2026,5,1),0),'Contract Data'!$F8&gt;=DATE(2026,5,1)),1,"")</f>
         <v/>
       </c>
-      <c r="W9" s="18">
+      <c r="W9" s="22">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2026,6,1),0),'Contract Data'!$F8&gt;=DATE(2026,6,1)),1,"")</f>
         <v/>
       </c>
-      <c r="X9" s="17">
+      <c r="X9" s="21">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2026,7,1),0),'Contract Data'!$F8&gt;=DATE(2026,7,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Y9" s="17">
+      <c r="Y9" s="21">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2026,8,1),0),'Contract Data'!$F8&gt;=DATE(2026,8,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Z9" s="17">
+      <c r="Z9" s="18">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2026,9,1),0),'Contract Data'!$F8&gt;=DATE(2026,9,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AA9" s="17">
+      <c r="AA9" s="18">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2026,10,1),0),'Contract Data'!$F8&gt;=DATE(2026,10,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AB9" s="17">
+      <c r="AB9" s="18">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2026,11,1),0),'Contract Data'!$F8&gt;=DATE(2026,11,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AC9" s="17">
+      <c r="AC9" s="18">
         <f>IF(AND('Contract Data'!$E8&lt;=EOMONTH(DATE(2026,12,1),0),'Contract Data'!$F8&gt;=DATE(2026,12,1)),1,"")</f>
         <v/>
       </c>
@@ -2108,99 +2114,99 @@
         <f>'Contract Data'!G9</f>
         <v/>
       </c>
-      <c r="F10" s="15">
+      <c r="F10" s="23">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2025,1,1),0),'Contract Data'!$F9&gt;=DATE(2025,1,1)),1,"")</f>
         <v/>
       </c>
-      <c r="G10" s="15">
+      <c r="G10" s="23">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2025,2,1),0),'Contract Data'!$F9&gt;=DATE(2025,2,1)),1,"")</f>
         <v/>
       </c>
-      <c r="H10" s="15">
+      <c r="H10" s="23">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2025,3,1),0),'Contract Data'!$F9&gt;=DATE(2025,3,1)),1,"")</f>
         <v/>
       </c>
-      <c r="I10" s="15">
+      <c r="I10" s="23">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2025,4,1),0),'Contract Data'!$F9&gt;=DATE(2025,4,1)),1,"")</f>
         <v/>
       </c>
-      <c r="J10" s="15">
+      <c r="J10" s="23">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2025,5,1),0),'Contract Data'!$F9&gt;=DATE(2025,5,1)),1,"")</f>
         <v/>
       </c>
-      <c r="K10" s="15">
+      <c r="K10" s="23">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2025,6,1),0),'Contract Data'!$F9&gt;=DATE(2025,6,1)),1,"")</f>
         <v/>
       </c>
-      <c r="L10" s="15">
+      <c r="L10" s="23">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2025,7,1),0),'Contract Data'!$F9&gt;=DATE(2025,7,1)),1,"")</f>
         <v/>
       </c>
-      <c r="M10" s="15">
+      <c r="M10" s="23">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2025,8,1),0),'Contract Data'!$F9&gt;=DATE(2025,8,1)),1,"")</f>
         <v/>
       </c>
-      <c r="N10" s="15">
+      <c r="N10" s="23">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2025,9,1),0),'Contract Data'!$F9&gt;=DATE(2025,9,1)),1,"")</f>
         <v/>
       </c>
-      <c r="O10" s="15">
+      <c r="O10" s="23">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2025,10,1),0),'Contract Data'!$F9&gt;=DATE(2025,10,1)),1,"")</f>
         <v/>
       </c>
-      <c r="P10" s="15">
+      <c r="P10" s="23">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2025,11,1),0),'Contract Data'!$F9&gt;=DATE(2025,11,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Q10" s="15">
+      <c r="Q10" s="23">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2025,12,1),0),'Contract Data'!$F9&gt;=DATE(2025,12,1)),1,"")</f>
         <v/>
       </c>
-      <c r="R10" s="15">
+      <c r="R10" s="16">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2026,1,1),0),'Contract Data'!$F9&gt;=DATE(2026,1,1)),1,"")</f>
         <v/>
       </c>
-      <c r="S10" s="15">
+      <c r="S10" s="16">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2026,2,1),0),'Contract Data'!$F9&gt;=DATE(2026,2,1)),1,"")</f>
         <v/>
       </c>
-      <c r="T10" s="15">
+      <c r="T10" s="16">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2026,3,1),0),'Contract Data'!$F9&gt;=DATE(2026,3,1)),1,"")</f>
         <v/>
       </c>
-      <c r="U10" s="15">
+      <c r="U10" s="16">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2026,4,1),0),'Contract Data'!$F9&gt;=DATE(2026,4,1)),1,"")</f>
         <v/>
       </c>
-      <c r="V10" s="15">
+      <c r="V10" s="16">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2026,5,1),0),'Contract Data'!$F9&gt;=DATE(2026,5,1)),1,"")</f>
         <v/>
       </c>
-      <c r="W10" s="16">
+      <c r="W10" s="17">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2026,6,1),0),'Contract Data'!$F9&gt;=DATE(2026,6,1)),1,"")</f>
         <v/>
       </c>
-      <c r="X10" s="15">
+      <c r="X10" s="16">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2026,7,1),0),'Contract Data'!$F9&gt;=DATE(2026,7,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Y10" s="15">
+      <c r="Y10" s="16">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2026,8,1),0),'Contract Data'!$F9&gt;=DATE(2026,8,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Z10" s="15">
+      <c r="Z10" s="16">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2026,9,1),0),'Contract Data'!$F9&gt;=DATE(2026,9,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AA10" s="15">
+      <c r="AA10" s="16">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2026,10,1),0),'Contract Data'!$F9&gt;=DATE(2026,10,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AB10" s="15">
+      <c r="AB10" s="16">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2026,11,1),0),'Contract Data'!$F9&gt;=DATE(2026,11,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AC10" s="15">
+      <c r="AC10" s="16">
         <f>IF(AND('Contract Data'!$E9&lt;=EOMONTH(DATE(2026,12,1),0),'Contract Data'!$F9&gt;=DATE(2026,12,1)),1,"")</f>
         <v/>
       </c>
@@ -2226,99 +2232,99 @@
         <f>'Contract Data'!G10</f>
         <v/>
       </c>
-      <c r="F11" s="17">
+      <c r="F11" s="18">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2025,1,1),0),'Contract Data'!$F10&gt;=DATE(2025,1,1)),1,"")</f>
         <v/>
       </c>
-      <c r="G11" s="17">
+      <c r="G11" s="18">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2025,2,1),0),'Contract Data'!$F10&gt;=DATE(2025,2,1)),1,"")</f>
         <v/>
       </c>
-      <c r="H11" s="17">
+      <c r="H11" s="18">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2025,3,1),0),'Contract Data'!$F10&gt;=DATE(2025,3,1)),1,"")</f>
         <v/>
       </c>
-      <c r="I11" s="17">
+      <c r="I11" s="18">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2025,4,1),0),'Contract Data'!$F10&gt;=DATE(2025,4,1)),1,"")</f>
         <v/>
       </c>
-      <c r="J11" s="17">
+      <c r="J11" s="23">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2025,5,1),0),'Contract Data'!$F10&gt;=DATE(2025,5,1)),1,"")</f>
         <v/>
       </c>
-      <c r="K11" s="17">
+      <c r="K11" s="23">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2025,6,1),0),'Contract Data'!$F10&gt;=DATE(2025,6,1)),1,"")</f>
         <v/>
       </c>
-      <c r="L11" s="17">
+      <c r="L11" s="23">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2025,7,1),0),'Contract Data'!$F10&gt;=DATE(2025,7,1)),1,"")</f>
         <v/>
       </c>
-      <c r="M11" s="17">
+      <c r="M11" s="23">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2025,8,1),0),'Contract Data'!$F10&gt;=DATE(2025,8,1)),1,"")</f>
         <v/>
       </c>
-      <c r="N11" s="17">
+      <c r="N11" s="23">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2025,9,1),0),'Contract Data'!$F10&gt;=DATE(2025,9,1)),1,"")</f>
         <v/>
       </c>
-      <c r="O11" s="17">
+      <c r="O11" s="23">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2025,10,1),0),'Contract Data'!$F10&gt;=DATE(2025,10,1)),1,"")</f>
         <v/>
       </c>
-      <c r="P11" s="17">
+      <c r="P11" s="23">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2025,11,1),0),'Contract Data'!$F10&gt;=DATE(2025,11,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Q11" s="17">
+      <c r="Q11" s="18">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2025,12,1),0),'Contract Data'!$F10&gt;=DATE(2025,12,1)),1,"")</f>
         <v/>
       </c>
-      <c r="R11" s="17">
+      <c r="R11" s="18">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2026,1,1),0),'Contract Data'!$F10&gt;=DATE(2026,1,1)),1,"")</f>
         <v/>
       </c>
-      <c r="S11" s="17">
+      <c r="S11" s="18">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2026,2,1),0),'Contract Data'!$F10&gt;=DATE(2026,2,1)),1,"")</f>
         <v/>
       </c>
-      <c r="T11" s="17">
+      <c r="T11" s="18">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2026,3,1),0),'Contract Data'!$F10&gt;=DATE(2026,3,1)),1,"")</f>
         <v/>
       </c>
-      <c r="U11" s="17">
+      <c r="U11" s="18">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2026,4,1),0),'Contract Data'!$F10&gt;=DATE(2026,4,1)),1,"")</f>
         <v/>
       </c>
-      <c r="V11" s="17">
+      <c r="V11" s="18">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2026,5,1),0),'Contract Data'!$F10&gt;=DATE(2026,5,1)),1,"")</f>
         <v/>
       </c>
-      <c r="W11" s="18">
+      <c r="W11" s="19">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2026,6,1),0),'Contract Data'!$F10&gt;=DATE(2026,6,1)),1,"")</f>
         <v/>
       </c>
-      <c r="X11" s="17">
+      <c r="X11" s="18">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2026,7,1),0),'Contract Data'!$F10&gt;=DATE(2026,7,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Y11" s="17">
+      <c r="Y11" s="18">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2026,8,1),0),'Contract Data'!$F10&gt;=DATE(2026,8,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Z11" s="17">
+      <c r="Z11" s="18">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2026,9,1),0),'Contract Data'!$F10&gt;=DATE(2026,9,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AA11" s="17">
+      <c r="AA11" s="18">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2026,10,1),0),'Contract Data'!$F10&gt;=DATE(2026,10,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AB11" s="17">
+      <c r="AB11" s="18">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2026,11,1),0),'Contract Data'!$F10&gt;=DATE(2026,11,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AC11" s="17">
+      <c r="AC11" s="18">
         <f>IF(AND('Contract Data'!$E10&lt;=EOMONTH(DATE(2026,12,1),0),'Contract Data'!$F10&gt;=DATE(2026,12,1)),1,"")</f>
         <v/>
       </c>
@@ -2344,99 +2350,99 @@
         <f>'Contract Data'!G11</f>
         <v/>
       </c>
-      <c r="F12" s="15">
+      <c r="F12" s="16">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2025,1,1),0),'Contract Data'!$F11&gt;=DATE(2025,1,1)),1,"")</f>
         <v/>
       </c>
-      <c r="G12" s="15">
+      <c r="G12" s="16">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2025,2,1),0),'Contract Data'!$F11&gt;=DATE(2025,2,1)),1,"")</f>
         <v/>
       </c>
-      <c r="H12" s="15">
+      <c r="H12" s="16">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2025,3,1),0),'Contract Data'!$F11&gt;=DATE(2025,3,1)),1,"")</f>
         <v/>
       </c>
-      <c r="I12" s="15">
+      <c r="I12" s="16">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2025,4,1),0),'Contract Data'!$F11&gt;=DATE(2025,4,1)),1,"")</f>
         <v/>
       </c>
-      <c r="J12" s="15">
+      <c r="J12" s="16">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2025,5,1),0),'Contract Data'!$F11&gt;=DATE(2025,5,1)),1,"")</f>
         <v/>
       </c>
-      <c r="K12" s="15">
+      <c r="K12" s="16">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2025,6,1),0),'Contract Data'!$F11&gt;=DATE(2025,6,1)),1,"")</f>
         <v/>
       </c>
-      <c r="L12" s="15">
+      <c r="L12" s="24">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2025,7,1),0),'Contract Data'!$F11&gt;=DATE(2025,7,1)),1,"")</f>
         <v/>
       </c>
-      <c r="M12" s="15">
+      <c r="M12" s="24">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2025,8,1),0),'Contract Data'!$F11&gt;=DATE(2025,8,1)),1,"")</f>
         <v/>
       </c>
-      <c r="N12" s="15">
+      <c r="N12" s="24">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2025,9,1),0),'Contract Data'!$F11&gt;=DATE(2025,9,1)),1,"")</f>
         <v/>
       </c>
-      <c r="O12" s="15">
+      <c r="O12" s="24">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2025,10,1),0),'Contract Data'!$F11&gt;=DATE(2025,10,1)),1,"")</f>
         <v/>
       </c>
-      <c r="P12" s="15">
+      <c r="P12" s="24">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2025,11,1),0),'Contract Data'!$F11&gt;=DATE(2025,11,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Q12" s="15">
+      <c r="Q12" s="24">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2025,12,1),0),'Contract Data'!$F11&gt;=DATE(2025,12,1)),1,"")</f>
         <v/>
       </c>
-      <c r="R12" s="15">
+      <c r="R12" s="24">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2026,1,1),0),'Contract Data'!$F11&gt;=DATE(2026,1,1)),1,"")</f>
         <v/>
       </c>
-      <c r="S12" s="15">
+      <c r="S12" s="24">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2026,2,1),0),'Contract Data'!$F11&gt;=DATE(2026,2,1)),1,"")</f>
         <v/>
       </c>
-      <c r="T12" s="15">
+      <c r="T12" s="24">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2026,3,1),0),'Contract Data'!$F11&gt;=DATE(2026,3,1)),1,"")</f>
         <v/>
       </c>
-      <c r="U12" s="15">
+      <c r="U12" s="24">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2026,4,1),0),'Contract Data'!$F11&gt;=DATE(2026,4,1)),1,"")</f>
         <v/>
       </c>
-      <c r="V12" s="15">
+      <c r="V12" s="24">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2026,5,1),0),'Contract Data'!$F11&gt;=DATE(2026,5,1)),1,"")</f>
         <v/>
       </c>
-      <c r="W12" s="16">
+      <c r="W12" s="25">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2026,6,1),0),'Contract Data'!$F11&gt;=DATE(2026,6,1)),1,"")</f>
         <v/>
       </c>
-      <c r="X12" s="15">
+      <c r="X12" s="16">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2026,7,1),0),'Contract Data'!$F11&gt;=DATE(2026,7,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Y12" s="15">
+      <c r="Y12" s="16">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2026,8,1),0),'Contract Data'!$F11&gt;=DATE(2026,8,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Z12" s="15">
+      <c r="Z12" s="16">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2026,9,1),0),'Contract Data'!$F11&gt;=DATE(2026,9,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AA12" s="15">
+      <c r="AA12" s="16">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2026,10,1),0),'Contract Data'!$F11&gt;=DATE(2026,10,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AB12" s="15">
+      <c r="AB12" s="16">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2026,11,1),0),'Contract Data'!$F11&gt;=DATE(2026,11,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AC12" s="15">
+      <c r="AC12" s="16">
         <f>IF(AND('Contract Data'!$E11&lt;=EOMONTH(DATE(2026,12,1),0),'Contract Data'!$F11&gt;=DATE(2026,12,1)),1,"")</f>
         <v/>
       </c>
@@ -2462,153 +2468,153 @@
         <f>'Contract Data'!G12</f>
         <v/>
       </c>
-      <c r="F13" s="17">
+      <c r="F13" s="18">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2025,1,1),0),'Contract Data'!$F12&gt;=DATE(2025,1,1)),1,"")</f>
         <v/>
       </c>
-      <c r="G13" s="17">
+      <c r="G13" s="18">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2025,2,1),0),'Contract Data'!$F12&gt;=DATE(2025,2,1)),1,"")</f>
         <v/>
       </c>
-      <c r="H13" s="17">
+      <c r="H13" s="18">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2025,3,1),0),'Contract Data'!$F12&gt;=DATE(2025,3,1)),1,"")</f>
         <v/>
       </c>
-      <c r="I13" s="17">
+      <c r="I13" s="18">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2025,4,1),0),'Contract Data'!$F12&gt;=DATE(2025,4,1)),1,"")</f>
         <v/>
       </c>
-      <c r="J13" s="17">
+      <c r="J13" s="18">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2025,5,1),0),'Contract Data'!$F12&gt;=DATE(2025,5,1)),1,"")</f>
         <v/>
       </c>
-      <c r="K13" s="17">
+      <c r="K13" s="18">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2025,6,1),0),'Contract Data'!$F12&gt;=DATE(2025,6,1)),1,"")</f>
         <v/>
       </c>
-      <c r="L13" s="17">
+      <c r="L13" s="18">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2025,7,1),0),'Contract Data'!$F12&gt;=DATE(2025,7,1)),1,"")</f>
         <v/>
       </c>
-      <c r="M13" s="17">
+      <c r="M13" s="18">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2025,8,1),0),'Contract Data'!$F12&gt;=DATE(2025,8,1)),1,"")</f>
         <v/>
       </c>
-      <c r="N13" s="17">
+      <c r="N13" s="18">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2025,9,1),0),'Contract Data'!$F12&gt;=DATE(2025,9,1)),1,"")</f>
         <v/>
       </c>
-      <c r="O13" s="17">
+      <c r="O13" s="24">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2025,10,1),0),'Contract Data'!$F12&gt;=DATE(2025,10,1)),1,"")</f>
         <v/>
       </c>
-      <c r="P13" s="17">
+      <c r="P13" s="24">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2025,11,1),0),'Contract Data'!$F12&gt;=DATE(2025,11,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Q13" s="17">
+      <c r="Q13" s="24">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2025,12,1),0),'Contract Data'!$F12&gt;=DATE(2025,12,1)),1,"")</f>
         <v/>
       </c>
-      <c r="R13" s="17">
+      <c r="R13" s="24">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2026,1,1),0),'Contract Data'!$F12&gt;=DATE(2026,1,1)),1,"")</f>
         <v/>
       </c>
-      <c r="S13" s="17">
+      <c r="S13" s="24">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2026,2,1),0),'Contract Data'!$F12&gt;=DATE(2026,2,1)),1,"")</f>
         <v/>
       </c>
-      <c r="T13" s="17">
+      <c r="T13" s="24">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2026,3,1),0),'Contract Data'!$F12&gt;=DATE(2026,3,1)),1,"")</f>
         <v/>
       </c>
-      <c r="U13" s="17">
+      <c r="U13" s="18">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2026,4,1),0),'Contract Data'!$F12&gt;=DATE(2026,4,1)),1,"")</f>
         <v/>
       </c>
-      <c r="V13" s="17">
+      <c r="V13" s="18">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2026,5,1),0),'Contract Data'!$F12&gt;=DATE(2026,5,1)),1,"")</f>
         <v/>
       </c>
-      <c r="W13" s="18">
+      <c r="W13" s="19">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2026,6,1),0),'Contract Data'!$F12&gt;=DATE(2026,6,1)),1,"")</f>
         <v/>
       </c>
-      <c r="X13" s="17">
+      <c r="X13" s="18">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2026,7,1),0),'Contract Data'!$F12&gt;=DATE(2026,7,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Y13" s="17">
+      <c r="Y13" s="18">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2026,8,1),0),'Contract Data'!$F12&gt;=DATE(2026,8,1)),1,"")</f>
         <v/>
       </c>
-      <c r="Z13" s="17">
+      <c r="Z13" s="18">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2026,9,1),0),'Contract Data'!$F12&gt;=DATE(2026,9,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AA13" s="17">
+      <c r="AA13" s="18">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2026,10,1),0),'Contract Data'!$F12&gt;=DATE(2026,10,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AB13" s="17">
+      <c r="AB13" s="18">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2026,11,1),0),'Contract Data'!$F12&gt;=DATE(2026,11,1)),1,"")</f>
         <v/>
       </c>
-      <c r="AC13" s="17">
+      <c r="AC13" s="18">
         <f>IF(AND('Contract Data'!$E12&lt;=EOMONTH(DATE(2026,12,1),0),'Contract Data'!$F12&gt;=DATE(2026,12,1)),1,"")</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="26" t="inlineStr">
         <is>
           <t>LEGEND</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="20" t="inlineStr"/>
-      <c r="B17" s="21" t="inlineStr">
+      <c r="A17" s="27" t="inlineStr"/>
+      <c r="B17" s="28" t="inlineStr">
         <is>
           <t>Acme Corp</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="22" t="inlineStr"/>
-      <c r="B18" s="21" t="inlineStr">
+      <c r="A18" s="29" t="inlineStr"/>
+      <c r="B18" s="28" t="inlineStr">
         <is>
           <t>Blue Ridge LLC</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="inlineStr"/>
-      <c r="B19" s="21" t="inlineStr">
+      <c r="A19" s="30" t="inlineStr"/>
+      <c r="B19" s="28" t="inlineStr">
         <is>
           <t>Summit Partners</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="24" t="inlineStr"/>
-      <c r="B20" s="21" t="inlineStr">
+      <c r="A20" s="31" t="inlineStr"/>
+      <c r="B20" s="28" t="inlineStr">
         <is>
           <t>Horizon Group</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="25" t="inlineStr"/>
-      <c r="B21" s="21" t="inlineStr">
+      <c r="A21" s="32" t="inlineStr"/>
+      <c r="B21" s="28" t="inlineStr">
         <is>
           <t>Crestview Inc</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="26" t="inlineStr"/>
-      <c r="B22" s="27" t="inlineStr">
+      <c r="A22" s="33" t="inlineStr"/>
+      <c r="B22" s="34" t="inlineStr">
         <is>
           <t>Today</t>
         </is>
@@ -2624,50 +2630,80 @@
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F4=1</formula>
     </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>F4=""</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F5:AC5">
-    <cfRule type="expression" priority="2" dxfId="0">
+    <cfRule type="expression" priority="3" dxfId="0">
       <formula>F5=1</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="2">
+      <formula>F5=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F6:AC6">
-    <cfRule type="expression" priority="3" dxfId="1">
+    <cfRule type="expression" priority="5" dxfId="3">
       <formula>F6=1</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="1">
+      <formula>F6=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F7:AC7">
-    <cfRule type="expression" priority="4" dxfId="1">
+    <cfRule type="expression" priority="7" dxfId="3">
       <formula>F7=1</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="2">
+      <formula>F7=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F8:AC8">
-    <cfRule type="expression" priority="5" dxfId="2">
+    <cfRule type="expression" priority="9" dxfId="4">
       <formula>F8=1</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="1">
+      <formula>F8=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F9:AC9">
-    <cfRule type="expression" priority="6" dxfId="2">
+    <cfRule type="expression" priority="11" dxfId="4">
       <formula>F9=1</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" dxfId="2">
+      <formula>F9=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F10:AC10">
-    <cfRule type="expression" priority="7" dxfId="3">
+    <cfRule type="expression" priority="13" dxfId="5">
       <formula>F10=1</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="1">
+      <formula>F10=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F11:AC11">
-    <cfRule type="expression" priority="8" dxfId="3">
+    <cfRule type="expression" priority="15" dxfId="5">
       <formula>F11=1</formula>
+    </cfRule>
+    <cfRule type="expression" priority="16" dxfId="2">
+      <formula>F11=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F12:AC12">
-    <cfRule type="expression" priority="9" dxfId="4">
+    <cfRule type="expression" priority="17" dxfId="6">
       <formula>F12=1</formula>
+    </cfRule>
+    <cfRule type="expression" priority="18" dxfId="1">
+      <formula>F12=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F13:AC13">
-    <cfRule type="expression" priority="10" dxfId="4">
+    <cfRule type="expression" priority="19" dxfId="6">
       <formula>F13=1</formula>
+    </cfRule>
+    <cfRule type="expression" priority="20" dxfId="2">
+      <formula>F13=""</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>